<commit_message>
Report and References update
</commit_message>
<xml_diff>
--- a/Modeling/Model_Result Summary.xlsx
+++ b/Modeling/Model_Result Summary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\vbshare2\PythonDA\LSTModels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\vbshare2\PythonDA\CT298ProjectDoc-main\Modeling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4991FED-BFB3-4D14-BCFF-AE6F7D30EC65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{790DA349-9757-4539-99CF-A9FC96643750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19305" yWindow="2415" windowWidth="18810" windowHeight="10305" activeTab="1" xr2:uid="{9CDB9373-15A7-4BB2-9A47-6CB38F4179DF}"/>
+    <workbookView xWindow="1240" yWindow="530" windowWidth="17810" windowHeight="9600" xr2:uid="{9CDB9373-15A7-4BB2-9A47-6CB38F4179DF}"/>
   </bookViews>
   <sheets>
     <sheet name="ARIMA" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="69">
   <si>
     <t>Ticker</t>
   </si>
@@ -157,9 +157,6 @@
     <t>9-20</t>
   </si>
   <si>
-    <t>21-2</t>
-  </si>
-  <si>
     <t>DA-DailyReturn</t>
   </si>
   <si>
@@ -236,6 +233,15 @@
   </si>
   <si>
     <t>apply GridSearchCV</t>
+  </si>
+  <si>
+    <t>22-3</t>
+  </si>
+  <si>
+    <t>build metrics to assess direction in prediction</t>
+  </si>
+  <si>
+    <t>LSTMwYFinance3ADirection</t>
   </si>
 </sst>
 </file>
@@ -344,7 +350,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -378,6 +384,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1205,14 +1214,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6115394-D851-4ADB-AC78-1E9CC5849655}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.796875" style="8" customWidth="1"/>
-    <col min="2" max="2" width="26.3984375" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="22.8984375" style="8" customWidth="1"/>
     <col min="4" max="4" width="8.796875" style="8"/>
-    <col min="5" max="5" width="39.59765625" customWidth="1"/>
+    <col min="5" max="5" width="42.69921875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.35">
@@ -1297,7 +1306,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>5</v>
@@ -1312,7 +1321,7 @@
         <v>33</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>36</v>
@@ -1327,7 +1336,7 @@
         <v>39</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>37</v>
@@ -1336,41 +1345,41 @@
         <v>3</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
-        <v>40</v>
+      <c r="A9" s="18">
+        <v>21</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="D9" s="9">
         <v>3</v>
       </c>
-      <c r="E9" s="12" t="s">
-        <v>65</v>
+      <c r="E9" s="10" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="9">
-        <v>23</v>
+      <c r="A10" s="9" t="s">
+        <v>66</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>37</v>
+        <v>59</v>
       </c>
       <c r="D10" s="9">
         <v>3</v>
       </c>
-      <c r="E10" s="10" t="s">
-        <v>66</v>
+      <c r="E10" s="12" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -1378,16 +1387,33 @@
         <v>24</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>62</v>
+        <v>37</v>
       </c>
       <c r="D11" s="9">
         <v>3</v>
       </c>
       <c r="E11" s="10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="9">
+        <v>25</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>63</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="D12" s="9">
+        <v>3</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
@@ -1426,25 +1452,25 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="C2" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="11" t="s">
         <v>47</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>48</v>
       </c>
       <c r="E2" s="10"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C3" s="9" t="s">
         <v>37</v>
@@ -1456,10 +1482,10 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>37</v>
@@ -1468,7 +1494,7 @@
         <v>3</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1507,40 +1533,40 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B2" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" s="11" t="s">
         <v>52</v>
-      </c>
-      <c r="C2" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>53</v>
       </c>
       <c r="E2" s="10"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C3" s="9" t="s">
         <v>36</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E3" s="10"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>37</v>
@@ -1555,10 +1581,10 @@
         <v>12</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D5" s="9">
         <v>3</v>

</xml_diff>